<commit_message>
Viewer: Street-View style look controls, all walls/tiles/doors/windows cut or hidden, transparent glass, sky, real mirror reflections, correct fabric/wall colours
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HKXAo1Q2bnBJX5nvnsockJ
</commit_message>
<xml_diff>
--- a/data/shopping.xlsx
+++ b/data/shopping.xlsx
@@ -7125,32 +7125,32 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Water heater 50 L</t>
+          <t>Water heater, flat 60 L, horizontal mounting</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Ariston Velis Pro 50 EU NEW (Technomarket 09242822)</t>
+          <t>Eldom Galant DU060W (60 L, 2.1+1.2 kW, universal mounting, el. control)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Ariston</t>
+          <t>Eldom</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>technomarket.bg</t>
+          <t>technika.bg</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>https://www.technomarket.bg/boiler/ariston-velis-pro-50-eu-new-09242822</t>
+          <t>https://technika.bg/product/27638/boyler-eldom-50-l-2-1kw-1-2kw-plosak-dizayn-universalen-montazh-el-upravlenie-emayliran-du060w.html</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>309.0</t>
+          <t>335.46</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -7160,7 +7160,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>51.1 W x 78.1 H x 27.0 D (horizontal: 78.1 wide x 51.1 high)</t>
+          <t>51.1 W x 83.8 H x 30 D (horizontal: 83.8 long x 51.1 high)</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -7170,7 +7170,7 @@
       </c>
       <c r="L109" t="inlineStr">
         <is>
-          <t>Current NEW version of the specified model; sale price (regular EUR 369); limited stock/last units incl. 2 Sofia stores; 1.5 kW; needs plumber + electrician (dedicated circuit)</t>
+          <t>also OVK Install 729 BGN</t>
         </is>
       </c>
     </row>

</xml_diff>